<commit_message>
This version updates the figure creation workflow to use the new approach implemented in `{ospsuite}` version 1x. See <link to documentation>
- Removed sheet "exportConfiguration" from the "Plots.xlsx" configuration. Automated export of figures generated from excel sheets to files is not supported any more. To export figures, use the standard `ggplot2`
- Removed class `ExportConfiguration` that was overriding `ExportConfiguration` from the `tlf` package.
- Removed function `createEsqlabsExportConfiguration()`
- Argument `outputFolder` removed from the signature of the function `createPlotsFromExcel()`
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/Plots.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/Plots.xlsx
@@ -1,25 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub repositories\ESQlabs\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FB839A-93D5-46E9-9467-F865FBA2C3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E158637-E132-43CF-9FDC-61990FF1E4D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="2" xr2:uid="{3D43716F-F01F-40EA-AEC2-E6E5F12B752F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="3" xr2:uid="{3D43716F-F01F-40EA-AEC2-E6E5F12B752F}"/>
   </bookViews>
   <sheets>
     <sheet name="DataCombined" sheetId="3" r:id="rId1"/>
     <sheet name="plotConfiguration" sheetId="9" r:id="rId2"/>
     <sheet name="plotGrids" sheetId="5" r:id="rId3"/>
-    <sheet name="exportConfiguration" sheetId="11" r:id="rId4"/>
-    <sheet name="dataTypes" sheetId="4" r:id="rId5"/>
-    <sheet name="plotTypes" sheetId="10" r:id="rId6"/>
-    <sheet name="ObservedDataNames" sheetId="12" r:id="rId7"/>
+    <sheet name="dataTypes" sheetId="4" r:id="rId4"/>
+    <sheet name="plotTypes" sheetId="10" r:id="rId5"/>
+    <sheet name="ObservedDataNames" sheetId="12" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="62">
   <si>
     <t>group</t>
   </si>
@@ -149,15 +148,6 @@
   </si>
   <si>
     <t>P3</t>
-  </si>
-  <si>
-    <t>plotGridName</t>
-  </si>
-  <si>
-    <t>outputName</t>
-  </si>
-  <si>
-    <t>width</t>
   </si>
   <si>
     <t>Aciclovir PVB</t>
@@ -632,13 +622,13 @@
         <v>22</v>
       </c>
       <c r="I1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="J1" t="s">
         <v>23</v>
       </c>
       <c r="K1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="L1" t="s">
         <v>24</v>
@@ -665,13 +655,13 @@
       </c>
       <c r="F2" s="2"/>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.4">
@@ -685,21 +675,21 @@
         <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -708,24 +698,24 @@
         <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s">
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -734,16 +724,16 @@
         <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H5">
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -812,25 +802,25 @@
         <v>14</v>
       </c>
       <c r="I1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="K1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="M1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.4">
@@ -844,16 +834,16 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="O2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.4">
@@ -867,7 +857,7 @@
         <v>19</v>
       </c>
       <c r="N3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.4">
@@ -883,22 +873,22 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="K5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="M5">
         <v>1.96</v>
@@ -938,7 +928,7 @@
         <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
@@ -946,18 +936,18 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
@@ -965,10 +955,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -977,32 +967,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C90A7A38-3099-4667-B241-E28D7B8B0B13}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="11.3828125" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="13.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.15234375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C15D6C-2CD2-47AE-90A6-7EE546C5950C}">
   <sheetPr codeName="Tabelle4"/>
   <dimension ref="A1:A3"/>
@@ -1028,7 +992,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8551BE5-7C15-4718-88B4-27F1A938F9CF}">
   <sheetPr codeName="Tabelle5"/>
   <dimension ref="A1:A6"/>
@@ -1069,7 +1033,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86F50EB7-9B8D-43C6-8095-37A547673E3C}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
@@ -1079,12 +1043,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1291,20 +1257,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCC0D355-BB44-49CE-BEA9-BF722D315860}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07DA2F2C-8C96-42F3-AA23-50DABD54D547}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
+    <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1329,12 +1296,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07DA2F2C-8C96-42F3-AA23-50DABD54D547}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCC0D355-BB44-49CE-BEA9-BF722D315860}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
-    <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Remove "export configuration" sheet from Plots excel
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/Plots.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/Plots.xlsx
@@ -1,25 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub repositories\ESQlabs\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FB839A-93D5-46E9-9467-F865FBA2C3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2E82D3-EC61-4D06-99C9-21A00AE20541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="2" xr2:uid="{3D43716F-F01F-40EA-AEC2-E6E5F12B752F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{3D43716F-F01F-40EA-AEC2-E6E5F12B752F}"/>
   </bookViews>
   <sheets>
     <sheet name="DataCombined" sheetId="3" r:id="rId1"/>
     <sheet name="plotConfiguration" sheetId="9" r:id="rId2"/>
     <sheet name="plotGrids" sheetId="5" r:id="rId3"/>
-    <sheet name="exportConfiguration" sheetId="11" r:id="rId4"/>
-    <sheet name="dataTypes" sheetId="4" r:id="rId5"/>
-    <sheet name="plotTypes" sheetId="10" r:id="rId6"/>
-    <sheet name="ObservedDataNames" sheetId="12" r:id="rId7"/>
+    <sheet name="dataTypes" sheetId="4" r:id="rId4"/>
+    <sheet name="plotTypes" sheetId="10" r:id="rId5"/>
+    <sheet name="ObservedDataNames" sheetId="12" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="62">
   <si>
     <t>group</t>
   </si>
@@ -149,15 +148,6 @@
   </si>
   <si>
     <t>P3</t>
-  </si>
-  <si>
-    <t>plotGridName</t>
-  </si>
-  <si>
-    <t>outputName</t>
-  </si>
-  <si>
-    <t>width</t>
   </si>
   <si>
     <t>Aciclovir PVB</t>
@@ -595,18 +585,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CF424A-768A-416F-94F0-2A05F47DDD9E}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultColWidth="10.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.53515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.15234375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.3046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.3828125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="73.3828125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="81.3046875" customWidth="1"/>
-    <col min="7" max="7" width="24.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="73.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="81.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -632,13 +622,13 @@
         <v>22</v>
       </c>
       <c r="I1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="J1" t="s">
         <v>23</v>
       </c>
       <c r="K1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="L1" t="s">
         <v>24</v>
@@ -647,7 +637,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -665,16 +655,16 @@
       </c>
       <c r="F2" s="2"/>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -685,21 +675,21 @@
         <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -708,24 +698,24 @@
         <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s">
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -734,16 +724,16 @@
         <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H5">
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -771,22 +761,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73B8908D-615D-4618-BFCF-D7DBA10892F0}">
   <sheetPr codeName="Tabelle2"/>
   <dimension ref="A1:O5"/>
-  <sheetFormatPr defaultColWidth="10.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.69140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.07421875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="5.69140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="9.3046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.3046875" customWidth="1"/>
-    <col min="14" max="14" width="12.15234375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" customWidth="1"/>
+    <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -812,28 +802,28 @@
         <v>14</v>
       </c>
       <c r="I1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="K1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="M1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -844,19 +834,19 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="O2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -867,10 +857,10 @@
         <v>19</v>
       </c>
       <c r="N3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -881,24 +871,24 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="K5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="M5">
         <v>1.96</v>
@@ -925,9 +915,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FF3CB29-E548-4DAF-A68B-014C6C094FDA}">
   <sheetPr codeName="Tabelle3"/>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="10.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -938,37 +928,37 @@
         <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -977,24 +967,24 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C90A7A38-3099-4667-B241-E28D7B8B0B13}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="11.3828125" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="13.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.15234375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C15D6C-2CD2-47AE-90A6-7EE546C5950C}">
+  <sheetPr codeName="Tabelle4"/>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" t="s">
-        <v>38</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1003,24 +993,39 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C15D6C-2CD2-47AE-90A6-7EE546C5950C}">
-  <sheetPr codeName="Tabelle4"/>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultColWidth="10.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8551BE5-7C15-4718-88B4-27F1A938F9CF}">
+  <sheetPr codeName="Tabelle5"/>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1029,62 +1034,23 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8551BE5-7C15-4718-88B4-27F1A938F9CF}">
-  <sheetPr codeName="Tabelle5"/>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultColWidth="11.3828125" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86F50EB7-9B8D-43C6-8095-37A547673E3C}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1291,20 +1257,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCC0D355-BB44-49CE-BEA9-BF722D315860}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07DA2F2C-8C96-42F3-AA23-50DABD54D547}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
+    <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1329,12 +1296,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07DA2F2C-8C96-42F3-AA23-50DABD54D547}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCC0D355-BB44-49CE-BEA9-BF722D315860}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
-    <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>